<commit_message>
added groupName on create user template (afilimon)
</commit_message>
<xml_diff>
--- a/UploadTemplates/addUserTemplate.xlsx
+++ b/UploadTemplates/addUserTemplate.xlsx
@@ -1,10 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="22527"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C00FD4F-8BD7-4188-B6A5-68B1A3AF7AA6}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
+    <workbookView xWindow="3030" yWindow="3030" windowWidth="16200" windowHeight="9360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="addUser" sheetId="1" r:id="rId1"/>
@@ -14,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>firstName</t>
   </si>
@@ -53,12 +54,15 @@
   </si>
   <si>
     <t>internalID</t>
+  </si>
+  <si>
+    <t>groupName</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -205,6 +209,23 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri" panose="020F0502020204030204"/>
@@ -240,6 +261,23 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -415,8 +453,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:N1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.28515625" customWidth="1"/>
@@ -432,9 +470,10 @@
     <col min="11" max="11" width="18.5703125" customWidth="1"/>
     <col min="12" max="12" width="22.5703125" customWidth="1"/>
     <col min="13" max="13" width="21.5703125" customWidth="1"/>
+    <col min="14" max="14" width="23.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>12</v>
       </c>
@@ -473,6 +512,9 @@
       </c>
       <c r="M1" s="1" t="s">
         <v>11</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
linked new user with role/group  on excel import (afilimon)
</commit_message>
<xml_diff>
--- a/UploadTemplates/addUserTemplate.xlsx
+++ b/UploadTemplates/addUserTemplate.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="22527"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C00FD4F-8BD7-4188-B6A5-68B1A3AF7AA6}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DDB9F1D-052E-4CF5-BE8A-265B83F16B9B}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3030" yWindow="3030" windowWidth="16200" windowHeight="9360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3375" yWindow="3375" windowWidth="16200" windowHeight="9360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="addUser" sheetId="1" r:id="rId1"/>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>firstName</t>
   </si>
@@ -57,6 +57,9 @@
   </si>
   <si>
     <t>groupName</t>
+  </si>
+  <si>
+    <t>roleName</t>
   </si>
 </sst>
 </file>
@@ -454,7 +457,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.28515625" customWidth="1"/>
@@ -471,9 +474,10 @@
     <col min="12" max="12" width="22.5703125" customWidth="1"/>
     <col min="13" max="13" width="21.5703125" customWidth="1"/>
     <col min="14" max="14" width="23.7109375" customWidth="1"/>
+    <col min="15" max="15" width="15.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>12</v>
       </c>
@@ -515,6 +519,9 @@
       </c>
       <c r="N1" s="1" t="s">
         <v>13</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>